<commit_message>
Replaced with excel sheet
</commit_message>
<xml_diff>
--- a/data/crackers_list.xlsx
+++ b/data/crackers_list.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Websites\Crackers_Ecommerce\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -4676,7 +4676,7 @@
         <v>0.25</v>
       </c>
       <c r="H130" s="5">
-        <f t="shared" ref="H130:H161" si="4">F130*(1-G130)</f>
+        <f t="shared" ref="H130:H131" si="4">F130*(1-G130)</f>
         <v>11250</v>
       </c>
     </row>

</xml_diff>